<commit_message>
update import users from excel example
</commit_message>
<xml_diff>
--- a/דוגמה לאקסל ייבוא אנשים.xlsx
+++ b/דוגמה לאקסל ייבוא אנשים.xlsx
@@ -1,46 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pandaunicorn/Downloads/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DFFE297-6E2A-8F4A-AE63-A0122D22E3CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16180" xr2:uid="{F8C5329A-AC90-3743-A73F-5BC038514749}"/>
+    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16180"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>שם מלא</t>
   </si>
   <si>
+    <t>טלפון</t>
+  </si>
+  <si>
     <t>ריק אסטלי</t>
   </si>
   <si>
@@ -50,20 +31,22 @@
     <t>ישראל ישראלי</t>
   </si>
   <si>
-    <t>טלפון</t>
+    <r>
+      <t>523456789</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -421,40 +404,40 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F09CA08D-5184-EB47-A393-4BED8248FE37}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="16" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" customHeight="1"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2">
         <v>521234567</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B3">
         <v>534565667</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>123456789</v>
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>